<commit_message>
make kpi_sheet the sheet that the workbook opens to
</commit_message>
<xml_diff>
--- a/notebooks/Performance Report - 2023Q1 - April – June 2023.xlsx
+++ b/notebooks/Performance Report - 2023Q1 - April – June 2023.xlsx
@@ -1074,17 +1074,17 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>$256,657.61</t>
+          <t>$442,154.72</t>
         </is>
       </c>
       <c r="B6" s="4" t="n"/>
       <c r="C6" s="4" t="n">
-        <v>42844</v>
+        <v>73285</v>
       </c>
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>$5.99</t>
+          <t>$6.03</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>98829.39999999999</v>
+        <v>171123.05</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>72266</v>
+        <v>124139.95</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1436,7 +1436,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>30477.15</v>
+        <v>51838.49</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>26723.5</v>
+        <v>45692.5</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1546,7 +1546,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14578.95</v>
+        <v>25506.3</v>
       </c>
       <c r="M6" t="n">
         <v>242</v>
@@ -1589,7 +1589,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4926</v>
+        <v>8681</v>
       </c>
       <c r="M7" t="n">
         <v>189</v>
@@ -1632,7 +1632,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4218.65</v>
+        <v>6994.95</v>
       </c>
       <c r="M8" t="n">
         <v>219</v>
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3076.8</v>
+        <v>5332</v>
       </c>
       <c r="M9" t="n">
         <v>231</v>
@@ -1718,7 +1718,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1561.16</v>
+        <v>2846.48</v>
       </c>
       <c r="M10" t="n">
         <v>191</v>
@@ -4719,7 +4719,7 @@
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Automated findings highlighting significant trends and patterns with identified areas for action.</t>
+          <t>Automated findings highlighting significant trends and patterns with identified areas for investigation.</t>
         </is>
       </c>
     </row>

</xml_diff>